<commit_message>
tc regr core 2
</commit_message>
<xml_diff>
--- a/TC001_Credentials.xlsx
+++ b/TC001_Credentials.xlsx
@@ -4,11 +4,11 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2436" windowWidth="17988" windowHeight="4380"/>
+    <workbookView xWindow="0" yWindow="2436" windowWidth="17988" windowHeight="4380" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="LoginCrendentials" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
+    <sheet name="Invalid Login Credentials" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -393,7 +393,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultColWidth="17" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.21875" style="1" customWidth="1"/>
@@ -416,29 +416,11 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A1" r:id="rId1"/>
     <hyperlink ref="A2" r:id="rId2"/>
     <hyperlink ref="B2" r:id="rId3"/>
-    <hyperlink ref="A3" r:id="rId4"/>
-    <hyperlink ref="A4" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -446,9 +428,34 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="25.44140625" customWidth="1"/>
+    <col min="2" max="2" width="20.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1"/>
+    <hyperlink ref="A1" r:id="rId2"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>